<commit_message>
Add John Deere green box to garage tracker
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AGgVVdEYAhwvi6FAdjy7Kz
</commit_message>
<xml_diff>
--- a/Garage_Items_Tracker.xlsx
+++ b/Garage_Items_Tracker.xlsx
@@ -718,13 +718,57 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="n"/>
-      <c r="H6" s="7" t="n"/>
+      <c r="A6" s="5" t="n">
+        <v>46316</v>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Green sheet-metal box (possible ballast/weight box or battery box) – floor rusted through at one end</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>John Deere (paint color; not confirmed)</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Parts only</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>Marketplace</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>FB Marketplace</t>
+        </is>
+      </c>
+      <c r="H6" s="7" t="n">
+        <v>30</v>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>Light iron / shred (if unsold)</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>To list</t>
+        </is>
+      </c>
       <c r="L6" s="7" t="n"/>
       <c r="M6" s="5" t="n"/>
       <c r="N6" s="8">
         <f>IF(L6="","",L6-H6)</f>
         <v/>
+      </c>
+      <c r="O6" s="6" t="inlineStr">
+        <is>
+          <t>ID unconfirmed: check for JD part # stamped inside/under, mounting brackets. Sell as JD box for restoration or rustic planter, $20–40. Scrap value only ~$1–3 (light iron). If no bites in 2–3 weeks, scrap with other steel.</t>
+        </is>
       </c>
     </row>
     <row r="7">

</xml_diff>